<commit_message>
feat : add inventory functions
인벤토리에 데이터 추가 및 제거 기능
</commit_message>
<xml_diff>
--- a/RPGProject/Assets/Project/Data/ExcelData/BuffInfo.xlsx
+++ b/RPGProject/Assets/Project/Data/ExcelData/BuffInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyb1\Documents\GitHub\RPG\RPGProject\Assets\Project\Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A5650A-420C-4EC3-B842-2757C8876D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB88772-6774-4AC8-8F11-C9A1B2F31024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6405" yWindow="4710" windowWidth="22965" windowHeight="11295" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
+    <workbookView xWindow="1230" yWindow="765" windowWidth="14790" windowHeight="10695" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="CSVEnums" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
data : Buff 및 effect data 수정
</commit_message>
<xml_diff>
--- a/RPGProject/Assets/Project/Data/ExcelData/BuffInfo.xlsx
+++ b/RPGProject/Assets/Project/Data/ExcelData/BuffInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyb1\Documents\GitHub\RPG\RPGProject\Assets\Project\Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB88772-6774-4AC8-8F11-C9A1B2F31024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDA3F59-C506-47BC-AD16-64F37CE34F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1230" yWindow="765" windowWidth="14790" windowHeight="10695" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
+    <workbookView xWindow="1965" yWindow="3600" windowWidth="14790" windowHeight="10695" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="CSVEnums" sheetId="1" r:id="rId1"/>

</xml_diff>